<commit_message>
refactor(truongnv): tái cấu trúc phân hệ Task 3-5, cập nhật báo cáo và dọn dẹp references
</commit_message>
<xml_diff>
--- a/workspaces/truongnv/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
+++ b/workspaces/truongnv/Meeting/PI_GUARD_PROCESS_REPORT.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,37 +30,43 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <i val="1"/>
       <color rgb="00E5E7EB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="11"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +103,12 @@
         <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,6 +169,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -921,214 +945,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BẢNG PHÂN RÃ CÔNG VIỆC &amp; NHẬT KÝ CHI TIẾT — NGUYỄN VĂN TRƯỜNG</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+          <t>BẢNG KẾ HOẠCH &amp; NHẬT KÝ CHI TIẾT CÁ NHÂN — NGUYỄN VĂN TRƯỜNG (NVTRUONGOPS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Mã SV: SE182034 | Trưởng nhóm (Leader) | Khóa luận Tốt nghiệp: PI-Guard | Cập nhật tự động từ Git Commit Log cá nhân (nvtruongops)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>I. KẾ HOẠCH PHÂN RÃ CÔNG VIỆC CỐT LÕI (LỘ TRÌNH 15 TUẦN HỌC KỲ FALL 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Mã Task</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Tuần / Giai Đoạn</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Nội Dung Công Việc Chi Tiết Của Trường</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Trạng Thái</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Sản Phẩm Đầu Ra (Artifacts)</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Hạn Chót</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Đánh Giá Cá Nhân</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>T01-NVT</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Tuần 1 (07/09 - 13/09)</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Họp khởi động GVHD (Meeting 1) &amp; Họp nhóm sàng lọc 10 papers khoa học (Meeting 2)</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Meeting 1 &amp; Meeting 2.md</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Đã chốt mục tiêu và sàng lọc 10 papers</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>T02-NVT</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Tuần 1 (07/09 - 13/09)</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Khảo sát và thu thập 17 bài báo IEEE/ACM &gt;= 2022 về LLM Security</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>References/REFERENCES_LOG.md</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>13/09/2026</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Đã lập ma trận liên kết 17 papers</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>T03-NVT</t>
+          <t>T01-NVT</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Tuần 2 (14/09 - 20/09)</t>
+          <t>Tuần 1 (07/09 - 13/09)</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Soạn thảo Chapter 1: Background, Problem Statement (Von Neumann NLP)</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Họp khởi động GVHD (Meeting 1-3) &amp; Họp nhóm sàng lọc 10 papers khoa học</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/chapters/01</t>
+          <t>Meeting 1, 2, 3.md &amp; Đăng ký đề tài</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Đang hoàn thiện phần bối cảnh</t>
+          <t>Đã chốt mục tiêu và sàng lọc 10 papers</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>T04-NVT</t>
+          <t>T02-NVT</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Tuần 2 (14/09 - 20/09)</t>
+          <t>Tuần 1 (07/09 - 13/09)</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Phân loại mối đe dọa (Threat Taxonomy: Direct/Indirect vs Jailbreak)</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Khảo sát và thu thập 18 bài báo IEEE/ACM &gt;= 2022 về LLM Security</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/thesis/</t>
+          <t>References/REFERENCES_LOG.md &amp; 18 PDFs</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Đã ánh xạ theo OWASP LLM01:2025</t>
+          <t>Đã lập ma trận liên kết và lưu trữ 18 PDFs</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>T05-NVT</t>
+          <t>T03-NVT</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1138,34 +1102,34 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Soạn thảo Chapter 2: Literature Review, SOTA Matrix &amp; Research Gaps</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Soạn thảo Chapter 1: Background, Problem Statement (Von Neumann NLP)</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/chapters/02</t>
+          <t>Final-Report/thesis/chapters/01_Introduction.md</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Đã phân tích SOTA ProtectAI, NeMo</t>
+          <t>Hoàn tất bối cảnh, 3 RQs và phạm vi</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>T06-NVT</t>
+          <t>T04-NVT</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1175,192 +1139,192 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Biên soạn Hồ sơ Kỹ thuật Review 1 &amp; Dàn ý Slide 9 trang thuyết trình</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Phân loại mối đe dọa (Threat Taxonomy: Direct/Indirect vs Jailbreak theo OWASP)</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>workspaces/truongnv/docs/thesis/</t>
+          <t>Final-Report/thesis/Review1_Problem_Definition.md</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Chuẩn bị kịch bản thuyết trình 15 phút</t>
+          <t>Ánh xạ 5D Framework &amp; NIST AI 100-2e2025</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>T07-NVT</t>
+          <t>T05-NVT</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Tuần 3 (21/09 - 27/09)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Điều phối hoàn thiện 2 chương, tổng kết và đồng bộ bản chính thức Review 1</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Đang thực hiện</t>
+          <t>Soạn thảo Chapter 2: Literature Review, SOTA Matrix &amp; Research Gaps</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>PI_GUARD_PROCESS_REPORT.xlsx</t>
+          <t>Final-Report/thesis/chapters/02_Literature_Review.md</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Họp cả 4 thành viên thống nhất</t>
+          <t>Khảo sát Guardrails SOTA và xác lập 3 Gaps</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>T08-NVT</t>
+          <t>T06-NVT</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Tuần 4 (28/09 - 04/10)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Chủ trì phần thuyết trình và BẢO VỆ REVIEW 1 TRƯỚC GVHD</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+          <t>Biên soạn Hồ sơ Kỹ thuật Review 1 &amp; Slide thuyết trình 22 trang gặp GVHD 10/09</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Biên bản nghiệm thu Review 1</t>
+          <t>reports/PI-GUARD-Present-109.pptx (22 slides)</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>04/10/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Bảo vệ thành công Chapter 1 &amp; 2</t>
+          <t>Thuyết trình và tiếp thu ý kiến GVHD</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>T09-NVT</t>
+          <t>T07-NVT</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
+          <t>Tuần 2 (14/09 - 20/09)</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Tải 5 bộ dataset từ Hugging Face &amp; viết thuật toán Group-Aware Split</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đồng quy tri thức tuần, biên dịch Master Thesis &amp; đồng bộ Docs Portal MkDocs</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>src/datasets/splitter.py</t>
+          <t>Final-Report/thesis/FINAL_THESIS.md &amp; Github-Page/</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>18/10/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Đảm bảo Jaccard similarity &lt; 0.15</t>
+          <t>Biên dịch 2 chương và xuất bản GitHub Pages</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>T10-NVT</t>
+          <t>T08-NVT</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
+          <t>Tuần 3 - 4 (21/09 - 04/10)</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Đánh giá phân phối nhãn, kiểm tra độ rò rỉ dữ liệu giữa Train/Val/Test</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+          <t>Chủ trì phần thuyết trình và BẢO VỆ REVIEW 1 TRƯỚC GVHD (REPORT NO.1 &amp; NO.2)</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Đang thực hiện</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>notebooks/01_dataset_analysis</t>
+          <t>Hồ sơ Review 1 &amp; Slide bảo vệ chính thức</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>18/10/2026</t>
+          <t>04/10/2026</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Tránh rò rỉ mẫu tương tự</t>
+          <t>Chuẩn bị diễn tập và rà soát hồ sơ</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>T11-NVT</t>
+          <t>T09-NVT</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Tuần 7 (19/10 - 25/10)</t>
+          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Soạn thảo, cập nhật docs Chapter 3 (Methodology - Report No.3) &amp; Slide Review 2</t>
+          <t>Tải 5 bộ dataset từ Hugging Face &amp; viết thuật toán Group-Aware Split</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1370,34 +1334,34 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>docs/thesis/chapters/03_Methodology.md</t>
+          <t>src/datasets/splitter.py &amp; manifests/</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>18/10/2026</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Chuẩn bị đầy đủ nội dung phương pháp luận</t>
+          <t>Đảm bảo Jaccard similarity &lt; 0.15</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>T12-NVT</t>
+          <t>T10-NVT</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Tuần 8 (26/10 - 01/11)</t>
+          <t>Tuần 5 - 6 (05/10 - 18/10)</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3), Nộp Report No.3 &amp; Cập nhật Docs</t>
+          <t>Đánh giá phân phối nhãn, kiểm tra độ rò rỉ dữ liệu giữa Train/Val/Test</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -1407,34 +1371,34 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Report No.3 &amp; Biên bản Review 2</t>
+          <t>notebooks/01_dataset_analysis</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>01/11/2026</t>
+          <t>18/10/2026</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Bảo vệ Review 2 và cập nhật docs theo góp ý</t>
+          <t>Tránh rò rỉ mẫu tương tự</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>T13-NVT</t>
+          <t>T11-NVT</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Tuần 9 - 12 (02/11 - 29/11)</t>
+          <t>Tuần 7 (19/10 - 25/10)</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Hỗ trợ thử nghiệm tối ưu Transformer &amp; tích hợp Prototype</t>
+          <t>Soạn thảo, cập nhật docs Chapter 3 (Methodology - Report No.3) &amp; Slide Review 2</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1444,34 +1408,34 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>models/ &amp; Chapter 4</t>
+          <t>docs/thesis/chapters/03_Methodology.md</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>29/11/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>Đo lường độ trễ trên CPU &amp; chuẩn bị demo</t>
+          <t>Chuẩn bị đầy đủ nội dung phương pháp luận</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>T14-NVT</t>
+          <t>T12-NVT</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Tuần 13 (30/11 - 06/12)</t>
+          <t>Tuần 8 (26/10 - 01/11)</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Điều phối kiểm thử tích hợp FastAPI Middleware &amp; BẢO VỆ HỘI ĐỒNG 1</t>
+          <t>BẢO VỆ REVIEW 2 TRƯỚC GVHD (CHAPTER 3), Nộp Report No.3 &amp; Cập nhật Docs</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -1481,34 +1445,34 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Hệ thống Prototype Demo &amp; Report No.4</t>
+          <t>Report No.3 &amp; Biên bản Review 2</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>06/12/2026</t>
+          <t>01/11/2026</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Bảo vệ Demo trước Hội đồng giữa kỳ Tuần 13</t>
+          <t>Bảo vệ Review 2 và cập nhật docs theo góp ý</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>T15-NVT</t>
+          <t>T13-NVT</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Tuần 14 (07/12 - 13/12)</t>
+          <t>Tuần 9 - 12 (02/11 - 29/11)</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Biên dịch toàn văn Master Thesis 6 chương qua script và quét Turnitin</t>
+          <t>Hỗ trợ thử nghiệm tối ưu Transformer &amp; tích hợp Prototype</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -1518,66 +1482,3512 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>docs/thesis/FINAL_THESIS.md</t>
+          <t>models/ &amp; Chapter 4</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>13/12/2026</t>
+          <t>29/11/2026</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Đảm bảo độ trùng lặp Turnitin &lt; 20%</t>
+          <t>Đo lường độ trễ trên CPU &amp; chuẩn bị demo</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
+          <t>T14-NVT</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 13 (30/11 - 06/12)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Điều phối kiểm thử tích hợp FastAPI Middleware &amp; BẢO VỆ HỘI ĐỒNG 1</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Hệ thống Prototype Demo &amp; Report No.4</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Bảo vệ Demo trước Hội đồng giữa kỳ Tuần 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>T15-NVT</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 14 (07/12 - 13/12)</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Biên dịch toàn văn Master Thesis 6 chương qua script và quét Turnitin</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>docs/thesis/FINAL_THESIS.md</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>13/12/2026</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Đảm bảo độ trùng lặp Turnitin &lt; 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
           <t>T16-NVT</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Tuần 15 (14/12 - 20/12)</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Chủ trì BẢO VỆ TỐT NGHIỆP CHÍNH THỨC TRƯỚC HỘI ĐỒNG FPT</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Slide Bảo vệ &amp; Đồ án hoàn chỉnh</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>20/12/2026</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Tốt nghiệp đạt điểm xuất sắc</t>
         </is>
       </c>
     </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>II. NHẬT KÝ CÔNG VIỆC THỰC TẾ CHI TIẾT THEO GIT COMMIT LOG (TÁC GIẢ: NVTRUONGOPS — 90 COMMITS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Mã Commit</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Thời Gian (Ngày &amp; Giờ)</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Nội Dung Kỹ Thuật Chi Tiết (Commit Message)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Trạng Thái</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Sản Phẩm Đầu Ra / Tệp Bàn Giao (Artifacts)</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Tuần / Cột Mốc</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Ghi Chú Kỹ Thuật &amp; Đánh Giá Kiểm Định</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>C01 [cd4cb95]</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01 18:33</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>feat: initial commit for PI-Guard capstone project</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>140 tệp (.agents/, .env.example, .github/...)</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>C02 [3a8f1d5]</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-01 18:34</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>docs: update repository links to nvtruongops/pi-guard in README</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>C03 [475c161]</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01 23:37</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>feat(governance): update Meeting 2 records, add workspace boundary audit tool and team git skills</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>56 tệp (.agents/, AGENTS.md, CONTRIBUTING.md...)</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>C04 [53a3d1d]</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-01 23:50</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>refactor(workspaces): simplify member folders to truongnv, ducnq, vietpmh, phuongddd and fix CI badge in README</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>70 tệp (.agents/, AGENTS.md, Meeting/...)</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>C05 [b175ac9]</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01 23:57</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>ci: fix ruff lint formatting, include data manifests, and verify test suite</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>24 tệp (.gitignore, data/, src/...)</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Cấu hình và kiểm thử bộ công cụ QA kiểm định chất lượng cục bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>C06 [a30ce0c]</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-02 00:05</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>chore(cleanup): centralize process report, hold future chapters, and clean workspaces</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>18 tệp (Meeting/, reports/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>C07 [23bb583]</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02 00:10</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>chore(data): hold root data directory until Review 2 and decouple CI evaluation</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>5 tệp (.github/, data/...)</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Cấu hình và kiểm thử bộ công cụ QA kiểm định chất lượng cục bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>C08 [9c0f4e8]</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-03 18:56</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>docs(truongnv): Update Review 1 threat model, model study guides, and MCP configs</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>14 tệp (.agents/, mcp.json, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>Tích hợp máy chủ MCP (OpenAlex, SemanticScholar, Kaggle) phục vụ nghiên cứu</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>C09 [c0f13c7]</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03 18:57</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>feat(docs): Setup MkDocs Material documentation portal and GitHub Pages deployment workflow</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>5 tệp (.github/, .gitignore, mkdocs.yml...)</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; xuất bản cổng tài liệu nghiên cứu MkDocs Material GitHub Pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>C10 [0948507]</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-03 19:18</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>fix(security): Remove internal confidential references and sanitize portal generation</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>4 tệp (.gitignore, docs/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>C11 [3ab8629]</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03 19:25</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>style(home): Redesign premium hero banner, metric indicators, and portal cards</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>mkdocs.yml, build_docs_portal.py</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; xuất bản cổng tài liệu nghiên cứu MkDocs Material GitHub Pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>C12 [5023ebc]</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-03 19:28</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>refactor(docs): Remove navigation tabs and simplify to minimalist documentation layout</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>mkdocs.yml, build_docs_portal.py</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>C13 [0155622]</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03 21:16</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>fix(docs): Audit and fix dead YouTube videos, paywalled DOI links, and add open-access paper references</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>6 tệp (Meeting/, scripts/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>C14 [8ed397f]</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-03 21:22</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>feat(governance): Enforce Resource and Literature Validation Protocol (Zero Dead Links &amp; Open-Access PDF Invariant)</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>4 tệp (.agents/, AGENTS.md, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>C15 [224cbb2]</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03 21:24</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>chore(audit): Refine URL audit script and polish skill documentation links</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>3 tệp (.agents/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm định chất lượng cục bộ, rà soát thuật ngữ học thuật nền tảng</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>C16 [df9b9d9]</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-03 21:27</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>feat(skills): Add resource-and-literature-validation skill with CLI tools and Open-Access resolution protocol</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>4 tệp (.agents/, AGENTS.md, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>C17 [f2769f9]</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 00:23</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>docs(tfidf): Refine academic description of Stanford IR Ch.6, Ch.11 and Cambridge TR-356</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>workspaces/truongnv/docs/model_study/01_tfidf_syntactic_baseline/resources_and_videos.md</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>C18 [ab4ad0a]</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 00:36</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>feat(docs): Add comprehensive attack study module covering Prompt Injection &amp; Modern Jailbreaks (DAN, Roleplay, VM, Cipher)</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>10 tệp (mkdocs.yml, scripts/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>Xây dựng Threat Taxonomy, phân loại Direct/Indirect PI &amp; Jailbreak theo OWASP</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>C19 [6278253]</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 01:07</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>docs(attack_study): Detail pre-2022 origins, expand 13 Prompt Injections &amp; 10 Jailbreak families with 26 Tencent operators</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>8 tệp (mkdocs.yml, scripts/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng Threat Taxonomy, phân loại Direct/Indirect PI &amp; Jailbreak theo OWASP</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>C20 [5c59a4d]</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 01:53</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>docs(attack_study): Ground every assertion in peer-reviewed literature with verified links</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>8 tệp (workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>C21 [02a3114]</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 02:15</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>docs(truongnv): ground 100% files in academic literature with zero dead links</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>19 tệp (scripts/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>C22 [1c2ead2]</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:13</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>feat(agents): learn academic grounding and citation anchor integrity rules and skills</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>4 tệp (.agents/, AGENTS.md...)</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>C23 [e612f3d]</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:18</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>feat(truongnv): add robustness on obfuscated and evasion study suite (leetspeak, base64, spacing)</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>7 tệp (mkdocs.yml, scripts/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Nghiên cứu &amp; kiểm thử độ bền đối kháng trước kỹ thuật làm mờ (Leetspeak, Base64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>C24 [1df8b71]</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:21</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>feat(tests): add automated empirical adversarial robustness tests and zero-width character stripping</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>cleaner.py, test_obfuscation_robustness.py</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G48" s="16" t="inlineStr">
+        <is>
+          <t>Nghiên cứu &amp; kiểm thử độ bền đối kháng trước kỹ thuật làm mờ (Leetspeak, Base64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>C25 [a7bfd29]</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:28</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>refactor(truongnv): remove duplicate FPT guidelines file and point to shared root docs</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>README.md, FPT_IAP491_Capstone_Guidelines_and_Rubrics_Summary.md</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>C26 [05a9d12]</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:38</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>feat(governance): reconfigure PROCESS_REPORT_CHECKLIST.md with detailed chronology from 29/08 kickoff and restore Sprint 1 TODO list</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>Meeting/PROCESS_REPORT_CHECKLIST.md</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G50" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>C27 [d09f99a]</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:43</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>feat(truongnv): add comprehensive Threat Modeling and Multi-Layer Defense study suite (Meeting 1 items 3 and 4)</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>8 tệp (mkdocs.yml, scripts/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>C28 [97da3fe]</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 03:49</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>feat(references): download and distribute screened papers to member workspaces and update Meeting 2 documentation</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>46 tệp (Meeting/, References/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G52" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>C29 [9ab25f5]</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 08:39</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>refactor(meeting): consolidate Sprint 1 TODO list into Meeting 1 and add 2-model research checklist in Meeting 2</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>7 tệp (Meeting/, mkdocs.yml, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>C30 [f25c7a2]</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 08:54</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>refactor(governance): standardize collaborative full-pipeline paradigm across all docs</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>17 tệp (.agents/, AGENTS.md, Meeting/...)</t>
+        </is>
+      </c>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>C31 [36cdfdd]</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:10</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>refactor(review1): ground review 1 scope to literature review and illustrative scenarios without premature empirical claims</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>14 tệp (Meeting/, reports/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>C32 [c639853]</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-04 09:18</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>refactor(ci): remove github workflows and enforce local-only validation suite</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>12 tệp (.agents/, .github/, AGENTS.md...)</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>Cấu hình và kiểm thử bộ công cụ QA kiểm định chất lượng cục bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>C33 [2bac269]</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-04 14:22</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>docs(meeting-thesis): update meeting notes, thesis guidelines, and sync references across workspaces</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>28 tệp (.agents/, AGENTS.md, Meeting/...)</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Sprint Tiền Đề (29/08 - 06/09)</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>C34 [f4ba113]</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:40</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>docs(reports): migrate supervisor progress presentation 10/09/2026, add meeting 3, unify process report and clean slide figures</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>53 tệp (.gitignore, CONTRIBUTING.md, Meeting/...)</t>
+        </is>
+      </c>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>C35 [38e3664]</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:17</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>fix(figures): eliminate duplicate figures, standardize 12 unique technical images, sync to reports/figures and align supervisor report</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>26 tệp (Meeting/, reports/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>Đồng quy tri thức tuần, biên dịch Master Thesis &amp; đồng bộ process report</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>C36 [d222661]</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:21</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>docs(meeting): update meeting 3 attendee roles, prune redundant sections, move FAQ to end of supervisor report</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>4 tệp (Meeting/, reports/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F60" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G60" s="16" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>C37 [11e10f2]</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:26</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>docs(truongnv): remove deprecated MEETING_1_AND_2_COMPLIANCE_AUDIT_REPORT</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>workspaces/truongnv/reports/MEETING_1_AND_2_COMPLIANCE_AUDIT_REPORT.md</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>C38 [2e4d67a]</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:32</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>docs(references): publish 8 supervisor slide foundational papers, sync REFERENCES_LOG to root repo and add Saltzer 1975 open-access PDF</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>7 tệp (References/, mkdocs.yml, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>C39 [6e7d65d]</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:47</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>refactor(structure): streamline root directories, group data/configs/models under notebooks, organize slide figures and simplify references docs</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>60 tệp (.agents/, .gitignore, README.md...)</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G63" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>C40 [8de19b8]</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:05</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>refactor(repo): consolidate repository architecture into 3 primary divisions: reports, workspaces, and docs for github pages</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>119 tệp (.agents/, .gitignore, AGENTS.md...)</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G64" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>C41 [62eb1cb]</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:11</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>refactor(repo): unify graduation thesis into reports/thesis as single source of truth and solidify 3-part architecture</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>17 tệp (.agents/, AGENTS.md, README.md...)</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>Soạn thảo &amp; cập nhật nội dung Luận văn (Chapters 1 &amp; 2), Threat Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>C42 [506c481]</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:17</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>refactor(architecture): reorganize repository into 3 primary divisions: Final-Report, Github-Page, and workspaces</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr">
+        <is>
+          <t>161 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G66" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>C43 [b15a6b5]</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:20</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>chore(scripts): align audit boundaries, gitignore, and benchmark defaults to Final-Report</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>5 tệp (.gitignore, Final-Report/, scripts/...)</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm định chất lượng cục bộ, rà soát thuật ngữ học thuật nền tảng</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>C44 [db6ea58]</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:33</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>refactor(architecture): consolidate src, tests, and scripts into Final-Report for strictly 3 root divisions</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t>58 tệp (.agents/, .gitignore, AGENTS.md...)</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G68" s="16" t="inlineStr">
+        <is>
+          <t>Tái cấu trúc repository theo chuẩn 3 phân hệ độc tôn của đồ án</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>C45 [0fedbe8]</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:55</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>refactor(config): encapsulate requirements and .env into Final-Report with root pointers</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>11 tệp (.env.example, Final-Report/, README.md...)</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>C46 [b992634]</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 00:58</t>
+        </is>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>refactor(root): streamline repository root by removing redundant config and requirements files</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t>7 tệp (.env.example, .vscode/, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G70" s="16" t="inlineStr">
+        <is>
+          <t>Tái cấu trúc repository theo chuẩn 3 phân hệ độc tôn của đồ án</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>C47 [1b41c82]</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:08</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>refactor(reports): consolidate periodic reports, presentation deck, and benchmark metrics into Final-Report/reports</t>
+        </is>
+      </c>
+      <c r="D71" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>17 tệp (.agents/, .gitignore, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>C48 [ee90b7e]</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:11</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>docs(readme): align with CAPSTONE PROJECT REGISTER, remove premature results and focal modules, mark quickstart coming soon</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>adversarial_benchmark.json, README.md</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G72" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>C49 [672e5f9]</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:17</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>chore(benchmark): update smoke test latency metrics</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Final-Report/reports/experiment_reports/adversarial_benchmark.json</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>C50 [c38f9eb]</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:51</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>fix(docs): resolve GitHub Pages 404, add deploy-docs workflow, and fix anchor integrity</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>6 tệp (.github/, Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G74" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>C51 [0270ea2]</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:57</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>refactor(repo): align README and enforce Review 1 zero-code invariant in Final-Report</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>53 tệp (Final-Report/, Github-Page/, README.md...)</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>C52 [a852916]</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:02</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>feat(arch): upgrade System Architecture in README and create docs-portal-sync-and-deploy skill</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>4 tệp (.agents/, AGENTS.md, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G76" s="16" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; xuất bản cổng tài liệu nghiên cứu MkDocs Material GitHub Pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>C53 [84c7e44]</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:05</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>docs(readme): streamline System Architecture and remove bloated config and bibliography sections</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>Tái cấu trúc repository theo chuẩn 3 phân hệ độc tôn của đồ án</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>C54 [bb2b67d]</t>
+        </is>
+      </c>
+      <c r="B78" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:10</t>
+        </is>
+      </c>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>chore(repo): reconstruct notebooks, dataset, src and tests scaffolding with readme and gitkeep</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>43 tệp (Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F78" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G78" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>C55 [43268ab]</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:16</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>docs(readme): fix architecture mermaid UI contrast, collapse thesis tree, and clean quickstart</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>Soạn thảo &amp; cập nhật nội dung Luận văn (Chapters 1 &amp; 2), Threat Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>C56 [ef9bed0]</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:21</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>docs(readme): convert to professional English standard and remove all emoji icons</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+      <c r="F80" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G80" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>C57 [ca81c2a]</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:26</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>docs(workflow): update CONTRIBUTING.md milestone plan and update CHANGELOG.md to 0.4.0</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>3 tệp (CHANGELOG.md, CONTRIBUTING.md, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>C58 [f24c517]</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:28</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>docs(portal): sanitize external relative links in docs portal builder and contributing guide</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>build_docs_portal.py, contributing_guide.md</t>
+        </is>
+      </c>
+      <c r="F82" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; xuất bản cổng tài liệu nghiên cứu MkDocs Material GitHub Pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>C59 [c2497c7]</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:39</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>docs(governance): align milestone timeline with FPT IAP491 guidelines and purge localhost URLs</t>
+        </is>
+      </c>
+      <c r="D83" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>4 tệp (CHANGELOG.md, CONTRIBUTING.md, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>C60 [b852f36]</t>
+        </is>
+      </c>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:49</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>docs(academic): standardize academic metadata (IA program, Fall 2026, purge Location) and designate supervisor Tran Van Ninh</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>13 tệp (CHANGELOG.md, Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F84" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G84" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>C61 [91e1ee6]</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:53</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>docs(governance): purge Git Feature Branch column from team allocation tables and sync documentation</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>17 tệp (AGENTS.md, CHANGELOG.md, CONTRIBUTING.md...)</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>C62 [e1a96d0]</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 02:57</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>docs(portal): purge fpt_capstone_guide from Github-Page portal and audit configs</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>5 tệp (CHANGELOG.md, Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F86" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G86" s="16" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; xuất bản cổng tài liệu nghiên cứu MkDocs Material GitHub Pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>C63 [9f557ff]</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 03:09</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>docs(governance): clarify internal guidelines confidentiality and Fall 2026 timeline independence</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>12 tệp (.agents/, AGENTS.md, CHANGELOG.md...)</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>C64 [6177928]</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 03:26</t>
+        </is>
+      </c>
+      <c r="C88" s="16" t="inlineStr">
+        <is>
+          <t>docs(scope): align academic research PoC scope and purge unverified supervisor title</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>13 tệp (.agents/, AGENTS.md, CHANGELOG.md...)</t>
+        </is>
+      </c>
+      <c r="F88" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G88" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>C65 [97958d9]</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 03:32</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>docs(governance): standardize AGENTS.md to English, sync mcp.json, add defense terminology blacklist, and update all 12 skills</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>AGENTS.md, team_governance.md</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G89" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>C66 [54e40da]</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 03:41</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>feat(mcp): add openalex, semanticscholar, and kaggle mcp servers for literature discovery and cloud gpu labs</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>3 tệp (.vscode/, AGENTS.md, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F90" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G90" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>C67 [a818701]</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 03:53</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>feat(references): standardize academic terminology and enrich REFERENCES_LOG with metadata and local-first protocol</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>37 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>C68 [2d28dd3]</t>
+        </is>
+      </c>
+      <c r="B92" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:07</t>
+        </is>
+      </c>
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>fix(references): rigorous fact-check audit across 18 core papers and supplementary literature</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t>3 tệp (Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F92" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G92" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>C69 [1b16b77]</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:13</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>refactor(references): finalize scientific precision across all 5 key critique points</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>REFERENCES_LOG.md, references_log.md</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G93" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>C70 [7e1e318]</t>
+        </is>
+      </c>
+      <c r="B94" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:21</t>
+        </is>
+      </c>
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>fix(references): refine literature matrix metadata, attribution, and naming standards</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E94" s="16" t="inlineStr">
+        <is>
+          <t>6 tệp (Final-Report/, Github-Page/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F94" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G94" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>C71 [6978b2a]</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:23</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>feat(governance): implement three-tier decoupling rules and academic paper rigor gate (/learn)</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>5 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G95" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>C72 [862eb8b]</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:31</t>
+        </is>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>docs(governance): implement four-tier provenance, modularize blacklist rule, and enforce academic humility</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>12 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F96" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G96" s="16" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>C73 [64c5e22]</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:39</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>docs(references): index all 25 local PDF files and synchronize literature matrix</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>3 tệp (Final-Report/, Github-Page/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>C74 [7044b0e]</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:45</t>
+        </is>
+      </c>
+      <c r="C98" s="16" t="inlineStr">
+        <is>
+          <t>docs(citations): harmonize paper metadata, titles, and venues across all thesis chapters and research dossiers</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E98" s="16" t="inlineStr">
+        <is>
+          <t>43 tệp (.agents/, Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G98" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>C75 [b27a53a]</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-10 04:50</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>docs(presentation): update Tencent paper citation and fix caption typo in PI-GUARD-Present-109.pptx</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>5 tệp (Final-Report/, Github-Page/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>C76 [c2a3beb]</t>
+        </is>
+      </c>
+      <c r="B100" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 21:03</t>
+        </is>
+      </c>
+      <c r="C100" s="16" t="inlineStr">
+        <is>
+          <t>chore(convergence): harmonize academic defense terminology, sync meeting 4 records, and update docs portal</t>
+        </is>
+      </c>
+      <c r="D100" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E100" s="16" t="inlineStr">
+        <is>
+          <t>109 tệp (CONTRIBUTING.md, Final-Report/, Github-Page/...)</t>
+        </is>
+      </c>
+      <c r="F100" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G100" s="16" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>C77 [9e64b77]</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:07</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>chore(governance): enforce anti-siloing invariant, modularize meeting 4 technical dossier, and sync process report</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>11 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F101" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G101" s="8" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa quy chế phân quyền, ranh giới thư mục &amp; tài liệu quản trị nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>C78 [d7963be]</t>
+        </is>
+      </c>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:20</t>
+        </is>
+      </c>
+      <c r="C102" s="16" t="inlineStr">
+        <is>
+          <t>docs(scorecard): harmonize executive scorecard with peer-reviewed citations, public code, datasets, and four-tier decoupling</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E102" s="16" t="inlineStr">
+        <is>
+          <t>5 tệp (workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F102" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G102" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="13" t="inlineStr">
+        <is>
+          <t>C79 [795aa19]</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:29</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>docs(scorecard): decouple methodology papers from benchmark datasets and clarify tier-2 single-model scope</t>
+        </is>
+      </c>
+      <c r="D103" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>workspaces/truongnv/reports/task_for_meeting_4/README.md</t>
+        </is>
+      </c>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G103" s="8" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>C80 [35d6a67]</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:39</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>refactor(truongnv): decouple Task 3 reference scorecard from Task 4 PI-Guard improvements</t>
+        </is>
+      </c>
+      <c r="D104" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>workspaces/truongnv/reports/task_for_meeting_4/README.md</t>
+        </is>
+      </c>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G104" s="16" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="13" t="inlineStr">
+        <is>
+          <t>C81 [cb4449f]</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:54</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>refactor(truongnv): align Model 2 as original DeBERTa-v3 FP32 in Task 3 and ground INT8 as Task 4 improvement</t>
+        </is>
+      </c>
+      <c r="D105" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>3 tệp (workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="inlineStr">
+        <is>
+          <t>Tái lập thực nghiệm mô hình DeBERTa-v3 PIGuard ACL 2025, đo latency &amp; F1</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>C82 [c61fbd1]</t>
+        </is>
+      </c>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:02</t>
+        </is>
+      </c>
+      <c r="C106" s="16" t="inlineStr">
+        <is>
+          <t>refactor(truongnv): ground Task 3 datasets strictly in referenced papers (AdvBench, Alpaca, DAN, BIPIA)</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>README.md, TASK_3_REPRODUCIBILITY_AND_DATASETS.md</t>
+        </is>
+      </c>
+      <c r="F106" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G106" s="16" t="inlineStr">
+        <is>
+          <t>Kiểm toán y văn, đồng bộ 18 bài báo cốt lõi &amp; liên kết Open-Access PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="13" t="inlineStr">
+        <is>
+          <t>C83 [4371b4d]</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:11</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>refactor(truongnv): streamline README.md scorecard to executive refer text and restructure reproduction protocol</t>
+        </is>
+      </c>
+      <c r="D107" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>README.md, TASK_3_REPRODUCIBILITY_AND_DATASETS.md</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
+          <t>Tái cấu trúc repository theo chuẩn 3 phân hệ độc tôn của đồ án</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>C84 [229d2b2]</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:16</t>
+        </is>
+      </c>
+      <c r="C108" s="16" t="inlineStr">
+        <is>
+          <t>style(truongnv): format markdown table and spacing in README.md</t>
+        </is>
+      </c>
+      <c r="D108" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t>workspaces/truongnv/reports/task_for_meeting_4/README.md</t>
+        </is>
+      </c>
+      <c r="F108" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G108" s="16" t="inlineStr">
+        <is>
+          <t>Cấu hình và kiểm thử bộ công cụ QA kiểm định chất lượng cục bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="13" t="inlineStr">
+        <is>
+          <t>C85 [2297215]</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:26</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>docs(truongnv): expand informal PI abbreviation to formal Prompt Injection in README.md</t>
+        </is>
+      </c>
+      <c r="D109" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>workspaces/truongnv/reports/task_for_meeting_4/README.md</t>
+        </is>
+      </c>
+      <c r="F109" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G109" s="8" t="inlineStr">
+        <is>
+          <t>Đã hoàn thành và kiểm tra hợp lệ trên nhánh main</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>C86 [80c128f]</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:31</t>
+        </is>
+      </c>
+      <c r="C110" s="16" t="inlineStr">
+        <is>
+          <t>docs(truongnv): enrich Task 1 and Task 2 with structured attack mechanisms, execution flows and impact analysis</t>
+        </is>
+      </c>
+      <c r="D110" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E110" s="16" t="inlineStr">
+        <is>
+          <t>3 tệp (workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F110" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G110" s="16" t="inlineStr">
+        <is>
+          <t>Xây dựng Threat Taxonomy, phân loại Direct/Indirect PI &amp; Jailbreak theo OWASP</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="13" t="inlineStr">
+        <is>
+          <t>C87 [743ca18]</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:39</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>docs(truongnv): upgrade Task 2 and skills to 5D Threat Analysis Framework</t>
+        </is>
+      </c>
+      <c r="D111" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E111" s="8" t="inlineStr">
+        <is>
+          <t>4 tệp (.agents/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng Threat Taxonomy, phân loại Direct/Indirect PI &amp; Jailbreak theo OWASP</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="14" t="inlineStr">
+        <is>
+          <t>C88 [5ac35af]</t>
+        </is>
+      </c>
+      <c r="B112" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-12 00:05</t>
+        </is>
+      </c>
+      <c r="C112" s="16" t="inlineStr">
+        <is>
+          <t>feat(truongnv): standardize academic terminology glossary and enrich Meeting 4 research tasks</t>
+        </is>
+      </c>
+      <c r="D112" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E112" s="16" t="inlineStr">
+        <is>
+          <t>27 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F112" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G112" s="16" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="13" t="inlineStr">
+        <is>
+          <t>C89 [fd9abd9]</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-12 03:29</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>docs(meeting4): decouple Task 1/2/3 from project model and consolidate PI-Guard improvements in Task 4</t>
+        </is>
+      </c>
+      <c r="D113" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E113" s="8" t="inlineStr">
+        <is>
+          <t>5 tệp (Final-Report/, workspaces/...)</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr">
+        <is>
+          <t>Tuần 1 (07/09 - 13/09)</t>
+        </is>
+      </c>
+      <c r="G113" s="8" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>C90 [4470298]</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:19</t>
+        </is>
+      </c>
+      <c r="C114" s="16" t="inlineStr">
+        <is>
+          <t>chore(sync): đồng bộ tài liệu Luận văn, Meeting 4-5, GitHub Pages và phân hệ tái lập PIGuard ACL 2025</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="E114" s="16" t="inlineStr">
+        <is>
+          <t>177 tệp (.agents/, AGENTS.md, Final-Report/...)</t>
+        </is>
+      </c>
+      <c r="F114" s="15" t="inlineStr">
+        <is>
+          <t>Tuần 2 (14/09 - 20/09)</t>
+        </is>
+      </c>
+      <c r="G114" s="16" t="inlineStr">
+        <is>
+          <t>Biên soạn biên bản họp, slide trình chiếu &amp; báo cáo tiến độ gặp GVHD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A23:G23"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:G4"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="D4:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Hoàn thành,Đang thực hiện,Chưa bắt đầu,Bị trễ"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>